<commit_message>
time update and paid
</commit_message>
<xml_diff>
--- a/misc/record/Time and Payment.xlsx
+++ b/misc/record/Time and Payment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bc3139/repo/work/Fortune500_SDG_Analysis/misc/record/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Documents/GitHub/Fortune500_SDG_Analysis/misc/record/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF398F8-0E0C-B542-B152-60AB3C8E9B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB49D5E-41E5-954D-83EA-3B7212485997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="760" windowWidth="29300" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="980" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
   <si>
     <t>Date</t>
   </si>
@@ -193,6 +193,33 @@
   </si>
   <si>
     <t>$530 (paid)</t>
+  </si>
+  <si>
+    <t>1 hour 20 mins</t>
+  </si>
+  <si>
+    <t>1 hour 30 mins</t>
+  </si>
+  <si>
+    <t>38 mins</t>
+  </si>
+  <si>
+    <t>1 hour</t>
+  </si>
+  <si>
+    <t>4 hour</t>
+  </si>
+  <si>
+    <t>3 hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 hour 20 mins (14 hour) </t>
+  </si>
+  <si>
+    <t>1500NTD = 48 USD</t>
+  </si>
+  <si>
+    <t>48*14=672</t>
   </si>
 </sst>
 </file>
@@ -343,7 +370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -375,7 +402,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1507,7 +1533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="6" width="12.6640625" style="1" customWidth="1"/>
@@ -3047,7 +3073,9 @@
       <c r="C102" s="29">
         <v>0.625</v>
       </c>
-      <c r="D102" s="31"/>
+      <c r="D102" s="30" t="s">
+        <v>28</v>
+      </c>
       <c r="E102" s="24"/>
     </row>
     <row r="103" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3060,7 +3088,9 @@
       <c r="C103" s="29">
         <v>0.625</v>
       </c>
-      <c r="D103" s="24"/>
+      <c r="D103" s="30" t="s">
+        <v>30</v>
+      </c>
       <c r="E103" s="24"/>
     </row>
     <row r="104" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3073,7 +3103,9 @@
       <c r="C104" s="29">
         <v>0.43055555555555558</v>
       </c>
-      <c r="D104" s="24"/>
+      <c r="D104" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="E104" s="24"/>
     </row>
     <row r="105" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3086,8 +3118,8 @@
       <c r="C105" s="24">
         <v>12</v>
       </c>
-      <c r="D105" s="24">
-        <v>1</v>
+      <c r="D105" s="30" t="s">
+        <v>30</v>
       </c>
       <c r="E105" s="24"/>
     </row>
@@ -3098,10 +3130,12 @@
       <c r="B106" s="29">
         <v>0.67361111111111116</v>
       </c>
-      <c r="C106" s="32">
+      <c r="C106" s="31">
         <v>0.70000000000000007</v>
       </c>
-      <c r="D106" s="24"/>
+      <c r="D106" s="30" t="s">
+        <v>29</v>
+      </c>
       <c r="E106" s="24"/>
     </row>
     <row r="107" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3114,7 +3148,9 @@
       <c r="C107" s="29">
         <v>0.9375</v>
       </c>
-      <c r="D107" s="24"/>
+      <c r="D107" s="30" t="s">
+        <v>28</v>
+      </c>
       <c r="E107" s="24"/>
     </row>
     <row r="108" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3127,7 +3163,9 @@
       <c r="C108" s="29">
         <v>0.79166666666666663</v>
       </c>
-      <c r="D108" s="24"/>
+      <c r="D108" s="30" t="s">
+        <v>31</v>
+      </c>
       <c r="E108" s="24"/>
     </row>
     <row r="109" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3140,8 +3178,72 @@
       <c r="C109" s="29">
         <v>0.47916666666666669</v>
       </c>
-      <c r="D109" s="24"/>
+      <c r="D109" s="30" t="s">
+        <v>32</v>
+      </c>
       <c r="E109" s="24"/>
+    </row>
+    <row r="110" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A110" s="24"/>
+      <c r="B110" s="24"/>
+      <c r="C110" s="24"/>
+      <c r="D110" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="E110" s="24"/>
+    </row>
+    <row r="111" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A111" s="24"/>
+      <c r="B111" s="24"/>
+      <c r="C111" s="24"/>
+      <c r="D111" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="E111" s="24"/>
+    </row>
+    <row r="112" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A112" s="24"/>
+      <c r="B112" s="24"/>
+      <c r="C112" s="24"/>
+      <c r="D112" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="E112" s="24"/>
+    </row>
+    <row r="113" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A113" s="24"/>
+      <c r="B113" s="24"/>
+      <c r="C113" s="24"/>
+      <c r="D113" s="24"/>
+      <c r="E113" s="24"/>
+    </row>
+    <row r="114" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A114" s="24"/>
+      <c r="B114" s="24"/>
+      <c r="C114" s="24"/>
+      <c r="D114" s="24"/>
+      <c r="E114" s="24"/>
+    </row>
+    <row r="115" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A115" s="24"/>
+      <c r="B115" s="24"/>
+      <c r="C115" s="24"/>
+      <c r="D115" s="24"/>
+      <c r="E115" s="24"/>
+    </row>
+    <row r="116" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A116" s="24"/>
+      <c r="B116" s="24"/>
+      <c r="C116" s="24"/>
+      <c r="D116" s="24"/>
+      <c r="E116" s="24"/>
+    </row>
+    <row r="117" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A117" s="24"/>
+      <c r="B117" s="24"/>
+      <c r="C117" s="24"/>
+      <c r="D117" s="24"/>
+      <c r="E117" s="24"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>